<commit_message>
Updated form estanterias  all logic
</commit_message>
<xml_diff>
--- a/standalone_apps/form_generator/templates/template-extintores-mlg.xlsx
+++ b/standalone_apps/form_generator/templates/template-extintores-mlg.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -138,6 +138,10 @@
       <name val="Arial"/>
       <family val="2"/>
       <sz val="16"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="8"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1810,7 +1814,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="392">
+  <cellXfs count="393">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="1"/>
@@ -2798,6 +2802,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -16825,7 +16832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ187"/>
+  <dimension ref="A1:AR187"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.796875" defaultRowHeight="13.2"/>
   <cols>
     <col width="4.19921875" customWidth="1" style="5" min="1" max="1"/>
@@ -20144,6 +20151,11 @@
       <c r="AO84" s="43" t="n"/>
       <c r="AP84" s="43" t="n"/>
       <c r="AQ84" s="44" t="n"/>
+      <c r="AR84" s="392" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="13.5" customHeight="1" s="185">
       <c r="A85" s="45" t="n"/>

</xml_diff>